<commit_message>
Updating the order sheet to include real costs.
</commit_message>
<xml_diff>
--- a/Charge_Indicator/BOM and Order Sheet/Order_Sheet.xlsx
+++ b/Charge_Indicator/BOM and Order Sheet/Order_Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nathanfikes/Documents/GitHub/AutoNav-Charge_Indicator-KiCad_Pcb/Charge_Indicator/BOM and Order Sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3316FE39-6571-8548-884E-81D0A765BFF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9072578-7390-B146-93FF-E887100355D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11000" yWindow="680" windowWidth="19240" windowHeight="18040" xr2:uid="{F977D430-13CE-AD47-96E5-85BBB755CDD5}"/>
+    <workbookView xWindow="11000" yWindow="680" windowWidth="19240" windowHeight="18020" xr2:uid="{F977D430-13CE-AD47-96E5-85BBB755CDD5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="166">
   <si>
     <t>Qty</t>
   </si>
@@ -523,13 +523,26 @@
   </si>
   <si>
     <t>https://jlcpcb.com/partdetail/TexasInstruments-BQ34Z100PWRR2/C7220642</t>
+  </si>
+  <si>
+    <t>Extra Costs</t>
+  </si>
+  <si>
+    <t>LCSC</t>
+  </si>
+  <si>
+    <t>Actual Costs Breakdown:</t>
+  </si>
+  <si>
+    <t>(Tariffs, Import Duties, Shipping, Etc, Change Suppliers)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
@@ -676,7 +689,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -686,45 +699,19 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -745,12 +732,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -760,6 +741,37 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1096,7 +1108,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5429AA39-1145-AF43-8726-DB045179E867}">
-  <dimension ref="A2:P40"/>
+  <dimension ref="A2:P46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" bestFit="1" customWidth="1"/>
@@ -1106,12 +1118,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="P2" s="33" t="s">
+      <c r="P2" s="21" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="64" x14ac:dyDescent="0.2">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="18" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1120,14 +1132,14 @@
       <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
       <c r="J3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1151,1300 +1163,1300 @@
       </c>
     </row>
     <row r="4" spans="1:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="30">
+      <c r="A4" s="18">
         <v>5</v>
       </c>
-      <c r="B4" s="23">
+      <c r="B4" s="13">
         <f>1*$A$4</f>
         <v>5</v>
       </c>
-      <c r="C4" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="14" t="s">
+      <c r="C4" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="17" t="s">
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="L4" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="M4" s="18" t="s">
+      <c r="K4" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="L4" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="24">
+      <c r="N4" s="14">
         <f>31.65/5</f>
         <v>6.33</v>
       </c>
-      <c r="O4" s="25">
+      <c r="O4" s="15">
         <f t="shared" ref="O4:O16" si="0">N4*B4</f>
         <v>31.65</v>
       </c>
-      <c r="P4" s="26" t="s">
+      <c r="P4" s="16" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B5" s="23">
+      <c r="B5" s="13">
         <f t="shared" ref="B5:B9" si="1">1*$A$4</f>
         <v>5</v>
       </c>
-      <c r="C5" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="14" t="s">
+      <c r="C5" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="17" t="s">
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="17" t="s">
+      <c r="K5" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="L5" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="M5" s="18" t="s">
+      <c r="L5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="N5" s="24">
+      <c r="N5" s="14">
         <v>0.1356</v>
       </c>
-      <c r="O5" s="25">
+      <c r="O5" s="15">
         <f t="shared" si="0"/>
         <v>0.67799999999999994</v>
       </c>
-      <c r="P5" s="27" t="s">
+      <c r="P5" s="17" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B6" s="23">
+      <c r="B6" s="13">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="14" t="s">
+      <c r="C6" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="17" t="s">
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="K6" s="17" t="s">
+      <c r="K6" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="L6" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="M6" s="18" t="s">
+      <c r="L6" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M6" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="N6" s="24">
+      <c r="N6" s="14">
         <v>0.14360000000000001</v>
       </c>
-      <c r="O6" s="25">
+      <c r="O6" s="15">
         <f t="shared" si="0"/>
         <v>0.71799999999999997</v>
       </c>
-      <c r="P6" s="27" t="s">
+      <c r="P6" s="17" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B7" s="23">
+      <c r="B7" s="13">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="C7" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="14" t="s">
+      <c r="C7" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="17" t="s">
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="K7" s="17" t="s">
+      <c r="K7" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="L7" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="M7" s="18" t="s">
+      <c r="L7" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M7" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="N7" s="24">
+      <c r="N7" s="14">
         <v>3.6200000000000003E-2</v>
       </c>
-      <c r="O7" s="25">
+      <c r="O7" s="15">
         <f t="shared" si="0"/>
         <v>0.18100000000000002</v>
       </c>
-      <c r="P7" s="27" t="s">
+      <c r="P7" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B8" s="23">
+      <c r="B8" s="13">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="14" t="s">
+      <c r="C8" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="17" t="s">
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="K8" s="17" t="s">
+      <c r="K8" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="L8" s="17" t="s">
+      <c r="L8" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="M8" s="18" t="s">
+      <c r="M8" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="N8" s="24">
+      <c r="N8" s="14">
         <v>0.45</v>
       </c>
-      <c r="O8" s="25">
+      <c r="O8" s="15">
         <f t="shared" si="0"/>
         <v>2.25</v>
       </c>
-      <c r="P8" s="27" t="s">
+      <c r="P8" s="17" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B9" s="23">
+      <c r="B9" s="13">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="C9" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="14" t="s">
+      <c r="C9" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="17" t="s">
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="K9" s="17" t="s">
+      <c r="K9" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="L9" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="M9" s="18" t="s">
+      <c r="L9" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M9" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="N9" s="24">
+      <c r="N9" s="14">
         <v>5.3E-3</v>
       </c>
-      <c r="O9" s="25">
+      <c r="O9" s="15">
         <f t="shared" si="0"/>
         <v>2.6499999999999999E-2</v>
       </c>
-      <c r="P9" s="27" t="s">
+      <c r="P9" s="17" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B10" s="23">
+      <c r="B10" s="13">
         <f>5*$A$4</f>
         <v>25</v>
       </c>
-      <c r="C10" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="14" t="s">
+      <c r="C10" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="17" t="s">
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="K10" s="17" t="s">
+      <c r="K10" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="L10" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="M10" s="18" t="s">
+      <c r="L10" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M10" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="N10" s="24">
+      <c r="N10" s="14">
         <v>5.1000000000000004E-3</v>
       </c>
-      <c r="O10" s="25">
+      <c r="O10" s="15">
         <f t="shared" si="0"/>
         <v>0.1275</v>
       </c>
-      <c r="P10" s="32" t="s">
+      <c r="P10" s="20" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B11" s="23">
+      <c r="B11" s="13">
         <f>8*$A$4</f>
         <v>40</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="14" t="s">
+      <c r="C11" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="17" t="s">
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="K11" s="17" t="s">
+      <c r="K11" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="L11" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="M11" s="18" t="s">
+      <c r="L11" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M11" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="N11" s="24">
+      <c r="N11" s="14">
         <v>5.4999999999999997E-3</v>
       </c>
-      <c r="O11" s="25">
+      <c r="O11" s="15">
         <f t="shared" si="0"/>
         <v>0.21999999999999997</v>
       </c>
-      <c r="P11" s="27" t="s">
+      <c r="P11" s="17" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B12" s="23">
+      <c r="B12" s="13">
         <f>3*$A$4</f>
         <v>15</v>
       </c>
-      <c r="C12" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" s="19" t="s">
+      <c r="C12" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="21"/>
-      <c r="J12" s="17" t="s">
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="25"/>
+      <c r="J12" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="K12" s="22" t="s">
+      <c r="K12" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="L12" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M12" s="18" t="s">
+      <c r="L12" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M12" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="N12" s="24">
+      <c r="N12" s="14">
         <v>4.5999999999999999E-3</v>
       </c>
-      <c r="O12" s="25">
+      <c r="O12" s="15">
         <f t="shared" si="0"/>
         <v>6.9000000000000006E-2</v>
       </c>
-      <c r="P12" s="27" t="s">
+      <c r="P12" s="17" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B13" s="23">
+      <c r="B13" s="13">
         <f>1*$A$4</f>
         <v>5</v>
       </c>
-      <c r="C13" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" s="19" t="s">
+      <c r="C13" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="21"/>
-      <c r="J13" s="22" t="s">
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="25"/>
+      <c r="J13" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="K13" s="22" t="s">
+      <c r="K13" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="L13" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M13" s="18" t="s">
+      <c r="L13" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M13" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="N13" s="24">
+      <c r="N13" s="14">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="O13" s="25">
+      <c r="O13" s="15">
         <f t="shared" si="0"/>
         <v>0.03</v>
       </c>
-      <c r="P13" s="27" t="s">
+      <c r="P13" s="17" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B14" s="23">
+      <c r="B14" s="13">
         <f>1*$A$4</f>
         <v>5</v>
       </c>
-      <c r="C14" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" s="19" t="s">
+      <c r="C14" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="21"/>
-      <c r="J14" s="17" t="s">
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="25"/>
+      <c r="J14" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="K14" s="22" t="s">
+      <c r="K14" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="L14" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M14" s="18" t="s">
+      <c r="L14" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M14" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="N14" s="24">
+      <c r="N14" s="14">
         <v>5.1000000000000004E-3</v>
       </c>
-      <c r="O14" s="25">
+      <c r="O14" s="15">
         <f t="shared" si="0"/>
         <v>2.5500000000000002E-2</v>
       </c>
-      <c r="P14" s="27" t="s">
+      <c r="P14" s="17" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B15" s="23">
+      <c r="B15" s="13">
         <f>1*$A$4</f>
         <v>5</v>
       </c>
-      <c r="C15" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" s="19" t="s">
+      <c r="C15" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="22" t="s">
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="K15" s="22" t="s">
+      <c r="K15" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="L15" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M15" s="18" t="s">
+      <c r="L15" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M15" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="N15" s="24">
+      <c r="N15" s="14">
         <v>4.7999999999999996E-3</v>
       </c>
-      <c r="O15" s="25">
+      <c r="O15" s="15">
         <f t="shared" si="0"/>
         <v>2.3999999999999997E-2</v>
       </c>
-      <c r="P15" s="27" t="s">
+      <c r="P15" s="17" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B16" s="23">
+      <c r="B16" s="13">
         <v>0</v>
       </c>
-      <c r="C16" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="19" t="s">
+      <c r="C16" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="21"/>
-      <c r="J16" s="22" t="s">
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="25"/>
+      <c r="J16" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="K16" s="22" t="s">
+      <c r="K16" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="L16" s="22" t="s">
+      <c r="L16" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="M16" s="18" t="s">
+      <c r="M16" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="N16" s="24">
+      <c r="N16" s="14">
         <v>0</v>
       </c>
-      <c r="O16" s="25">
+      <c r="O16" s="15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="P16" s="18" t="s">
+      <c r="P16" s="11" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="17" spans="2:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B17" s="23">
+      <c r="B17" s="13">
         <f>1*$A$4</f>
         <v>5</v>
       </c>
-      <c r="C17" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="14" t="s">
+      <c r="C17" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="17" t="s">
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="28"/>
+      <c r="J17" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="K17" s="17" t="s">
+      <c r="K17" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="L17" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="M17" s="34" t="s">
+      <c r="L17" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M17" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="N17" s="24">
+      <c r="N17" s="14">
         <v>0.21560000000000001</v>
       </c>
-      <c r="O17" s="25">
+      <c r="O17" s="15">
         <f t="shared" ref="O17:O30" si="2">N17*B17</f>
         <v>1.0780000000000001</v>
       </c>
-      <c r="P17" s="32" t="s">
+      <c r="P17" s="20" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="18" spans="2:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B18" s="23">
+      <c r="B18" s="13">
         <f>2*$A$4</f>
         <v>10</v>
       </c>
-      <c r="C18" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" s="14" t="s">
+      <c r="C18" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="17" t="s">
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="K18" s="17" t="s">
+      <c r="K18" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="L18" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="M18" s="18" t="s">
+      <c r="L18" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M18" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="N18" s="24">
+      <c r="N18" s="14">
         <v>4.2500000000000003E-2</v>
       </c>
-      <c r="O18" s="25">
+      <c r="O18" s="15">
         <f t="shared" si="2"/>
         <v>0.42500000000000004</v>
       </c>
-      <c r="P18" s="27" t="s">
+      <c r="P18" s="17" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="19" spans="2:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B19" s="23">
+      <c r="B19" s="13">
         <f>2*$A$4</f>
         <v>10</v>
       </c>
-      <c r="C19" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="19" t="s">
+      <c r="C19" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="22" t="s">
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="24"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="K19" s="22" t="s">
+      <c r="K19" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="L19" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M19" s="34" t="s">
+      <c r="L19" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M19" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="N19" s="24">
+      <c r="N19" s="14">
         <v>2.1600000000000001E-2</v>
       </c>
-      <c r="O19" s="25">
+      <c r="O19" s="15">
         <f t="shared" si="2"/>
         <v>0.21600000000000003</v>
       </c>
-      <c r="P19" s="27" t="s">
+      <c r="P19" s="17" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B20" s="23">
+      <c r="B20" s="13">
         <f>1*$A$4</f>
         <v>5</v>
       </c>
-      <c r="C20" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" s="19" t="s">
+      <c r="C20" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="22" t="s">
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="K20" s="22" t="s">
+      <c r="K20" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="L20" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M20" s="18" t="s">
+      <c r="L20" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M20" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="N20" s="24">
+      <c r="N20" s="14">
         <v>0.113</v>
       </c>
-      <c r="O20" s="25">
+      <c r="O20" s="15">
         <f t="shared" si="2"/>
         <v>0.56500000000000006</v>
       </c>
-      <c r="P20" s="27" t="s">
+      <c r="P20" s="17" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="21" spans="2:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B21" s="23">
+      <c r="B21" s="13">
         <f>2*$A$4</f>
         <v>10</v>
       </c>
-      <c r="C21" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D21" s="19" t="s">
+      <c r="C21" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="17" t="s">
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="25"/>
+      <c r="J21" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="K21" s="22" t="s">
+      <c r="K21" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="L21" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M21" s="18" t="s">
+      <c r="L21" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M21" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="N21" s="24">
+      <c r="N21" s="14">
         <v>0.1148</v>
       </c>
-      <c r="O21" s="25">
+      <c r="O21" s="15">
         <f t="shared" si="2"/>
         <v>1.1479999999999999</v>
       </c>
-      <c r="P21" s="27" t="s">
+      <c r="P21" s="17" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B22" s="23">
+      <c r="B22" s="13">
         <f>1*$A$4</f>
         <v>5</v>
       </c>
-      <c r="C22" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" s="19" t="s">
+      <c r="C22" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="E22" s="20"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="20"/>
-      <c r="H22" s="20"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="22" t="s">
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="25"/>
+      <c r="J22" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="K22" s="22" t="s">
+      <c r="K22" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="L22" s="22" t="s">
+      <c r="L22" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="M22" s="18" t="s">
+      <c r="M22" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="N22" s="24">
+      <c r="N22" s="14">
         <v>2.2200000000000002</v>
       </c>
-      <c r="O22" s="25">
+      <c r="O22" s="15">
         <f t="shared" si="2"/>
         <v>11.100000000000001</v>
       </c>
-      <c r="P22" s="27" t="s">
+      <c r="P22" s="17" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="23" spans="2:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B23" s="23">
+      <c r="B23" s="13">
         <f>1*$A$4</f>
         <v>5</v>
       </c>
-      <c r="C23" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D23" s="19" t="s">
+      <c r="C23" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="21"/>
-      <c r="J23" s="17" t="s">
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="25"/>
+      <c r="J23" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="K23" s="17" t="s">
+      <c r="K23" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="L23" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M23" s="18" t="s">
+      <c r="L23" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M23" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="N23" s="24">
+      <c r="N23" s="14">
         <v>3.7100000000000001E-2</v>
       </c>
-      <c r="O23" s="25">
+      <c r="O23" s="15">
         <f t="shared" si="2"/>
         <v>0.1855</v>
       </c>
-      <c r="P23" s="27" t="s">
+      <c r="P23" s="17" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="24" spans="2:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B24" s="23">
+      <c r="B24" s="13">
         <f>3*$A$4</f>
         <v>15</v>
       </c>
-      <c r="C24" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" s="14" t="s">
+      <c r="C24" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="26" t="s">
         <v>110</v>
       </c>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
-      <c r="I24" s="16"/>
-      <c r="J24" s="17" t="s">
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="28"/>
+      <c r="J24" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="K24" s="17" t="s">
+      <c r="K24" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="L24" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="M24" s="18" t="s">
+      <c r="L24" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M24" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="N24" s="24">
+      <c r="N24" s="14">
         <v>2.9100000000000001E-2</v>
       </c>
-      <c r="O24" s="25">
+      <c r="O24" s="15">
         <f t="shared" si="2"/>
         <v>0.4365</v>
       </c>
-      <c r="P24" s="27" t="s">
+      <c r="P24" s="17" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="25" spans="2:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B25" s="23">
+      <c r="B25" s="13">
         <f>1*$A$4</f>
         <v>5</v>
       </c>
-      <c r="C25" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D25" s="14" t="s">
+      <c r="C25" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="26" t="s">
         <v>115</v>
       </c>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="17" t="s">
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
+      <c r="I25" s="28"/>
+      <c r="J25" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="K25" s="17" t="s">
+      <c r="K25" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="L25" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="M25" s="18" t="s">
+      <c r="L25" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M25" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="N25" s="24">
+      <c r="N25" s="14">
         <v>0.62549999999999994</v>
       </c>
-      <c r="O25" s="25">
+      <c r="O25" s="15">
         <f t="shared" si="2"/>
         <v>3.1274999999999995</v>
       </c>
-      <c r="P25" s="27" t="s">
+      <c r="P25" s="17" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="26" spans="2:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B26" s="23">
-        <f t="shared" ref="B26:B42" si="3">1*$A$4</f>
+      <c r="B26" s="13">
+        <f t="shared" ref="B26:B36" si="3">1*$A$4</f>
         <v>5</v>
       </c>
-      <c r="C26" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D26" s="19" t="s">
+      <c r="C26" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="20"/>
-      <c r="H26" s="20"/>
-      <c r="I26" s="21"/>
-      <c r="J26" s="17" t="s">
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="25"/>
+      <c r="J26" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="K26" s="22" t="s">
+      <c r="K26" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="L26" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M26" s="18" t="s">
+      <c r="L26" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M26" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="N26" s="24">
+      <c r="N26" s="14">
         <v>0.27739999999999998</v>
       </c>
-      <c r="O26" s="25">
+      <c r="O26" s="15">
         <f t="shared" si="2"/>
         <v>1.387</v>
       </c>
-      <c r="P26" s="27" t="s">
+      <c r="P26" s="17" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B27" s="23">
+      <c r="B27" s="13">
         <f>2*$A$4</f>
         <v>10</v>
       </c>
-      <c r="C27" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" s="19" t="s">
+      <c r="C27" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="20"/>
-      <c r="I27" s="21"/>
-      <c r="J27" s="22" t="s">
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="25"/>
+      <c r="J27" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="K27" s="22" t="s">
+      <c r="K27" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="L27" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M27" s="18" t="s">
+      <c r="L27" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M27" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="N27" s="24">
+      <c r="N27" s="14">
         <v>0.15770000000000001</v>
       </c>
-      <c r="O27" s="25">
+      <c r="O27" s="15">
         <f t="shared" si="2"/>
         <v>1.577</v>
       </c>
-      <c r="P27" s="32" t="s">
+      <c r="P27" s="20" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="28" spans="2:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B28" s="23">
+      <c r="B28" s="13">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="C28" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D28" s="19" t="s">
+      <c r="C28" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" s="23" t="s">
         <v>125</v>
       </c>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="20"/>
-      <c r="I28" s="21"/>
-      <c r="J28" s="17" t="s">
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="K28" s="22" t="s">
+      <c r="K28" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="L28" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M28" s="18" t="s">
+      <c r="L28" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M28" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="N28" s="24">
+      <c r="N28" s="14">
         <v>4.1000000000000002E-2</v>
       </c>
-      <c r="O28" s="25">
+      <c r="O28" s="15">
         <f t="shared" si="2"/>
         <v>0.20500000000000002</v>
       </c>
-      <c r="P28" s="27" t="s">
+      <c r="P28" s="17" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B29" s="23">
+      <c r="B29" s="13">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="C29" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D29" s="19" t="s">
+      <c r="C29" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="E29" s="20"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="20"/>
-      <c r="H29" s="20"/>
-      <c r="I29" s="21"/>
-      <c r="J29" s="22" t="s">
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="24"/>
+      <c r="H29" s="24"/>
+      <c r="I29" s="25"/>
+      <c r="J29" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="K29" s="22" t="s">
+      <c r="K29" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="L29" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M29" s="18" t="s">
+      <c r="L29" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M29" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="N29" s="24">
+      <c r="N29" s="14">
         <v>3.5299999999999998E-2</v>
       </c>
-      <c r="O29" s="25">
+      <c r="O29" s="15">
         <f t="shared" si="2"/>
         <v>0.17649999999999999</v>
       </c>
-      <c r="P29" s="32" t="s">
+      <c r="P29" s="20" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="30" spans="2:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B30" s="23">
+      <c r="B30" s="13">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="C30" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D30" s="19" t="s">
+      <c r="C30" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="E30" s="20"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="20"/>
-      <c r="H30" s="20"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="17" t="s">
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="25"/>
+      <c r="J30" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="K30" s="22" t="s">
+      <c r="K30" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="L30" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M30" s="18" t="s">
+      <c r="L30" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M30" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="N30" s="24">
+      <c r="N30" s="14">
         <v>4.8500000000000001E-2</v>
       </c>
-      <c r="O30" s="25">
+      <c r="O30" s="15">
         <f t="shared" si="2"/>
         <v>0.24249999999999999</v>
       </c>
-      <c r="P30" s="27" t="s">
+      <c r="P30" s="17" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="31" spans="2:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B31" s="23">
+      <c r="B31" s="13">
         <f>7*$A$4</f>
         <v>35</v>
       </c>
-      <c r="C31" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D31" s="14" t="s">
+      <c r="C31" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="E31" s="15"/>
-      <c r="F31" s="15"/>
-      <c r="G31" s="15"/>
-      <c r="H31" s="15"/>
-      <c r="I31" s="16"/>
-      <c r="J31" s="17" t="s">
+      <c r="E31" s="27"/>
+      <c r="F31" s="27"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="28"/>
+      <c r="J31" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="K31" s="17" t="s">
+      <c r="K31" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="L31" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="M31" s="18" t="s">
+      <c r="L31" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="M31" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="N31" s="24">
+      <c r="N31" s="14">
         <v>3.4099999999999998E-2</v>
       </c>
-      <c r="O31" s="25">
-        <f t="shared" ref="O31:O42" si="4">N31*B31</f>
+      <c r="O31" s="15">
+        <f t="shared" ref="O31:O36" si="4">N31*B31</f>
         <v>1.1935</v>
       </c>
-      <c r="P31" s="27" t="s">
+      <c r="P31" s="17" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="32" spans="2:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B32" s="23">
+      <c r="B32" s="13">
         <f>2*$A$4</f>
         <v>10</v>
       </c>
-      <c r="C32" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D32" s="19" t="s">
+      <c r="C32" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D32" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="E32" s="20"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="20"/>
-      <c r="H32" s="20"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="22">
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="12">
         <v>1711725</v>
       </c>
-      <c r="K32" s="17" t="s">
+      <c r="K32" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="L32" s="22" t="s">
+      <c r="L32" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="M32" s="18" t="s">
+      <c r="M32" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="N32" s="24">
+      <c r="N32" s="14">
         <v>1.6879999999999999</v>
       </c>
-      <c r="O32" s="25">
+      <c r="O32" s="15">
         <f t="shared" si="4"/>
         <v>16.88</v>
       </c>
-      <c r="P32" s="27" t="s">
+      <c r="P32" s="17" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="33" spans="2:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="B33" s="23">
+      <c r="B33" s="13">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="C33" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D33" s="19" t="s">
+      <c r="C33" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="20"/>
-      <c r="H33" s="20"/>
-      <c r="I33" s="21"/>
-      <c r="J33" s="22" t="s">
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="25"/>
+      <c r="J33" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="K33" s="17" t="s">
+      <c r="K33" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="L33" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M33" s="18" t="s">
+      <c r="L33" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M33" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="N33" s="24">
+      <c r="N33" s="14">
         <v>0.15049999999999999</v>
       </c>
-      <c r="O33" s="25">
+      <c r="O33" s="15">
         <f t="shared" si="4"/>
         <v>0.75249999999999995</v>
       </c>
-      <c r="P33" s="27" t="s">
+      <c r="P33" s="17" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="34" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B34" s="23">
+      <c r="B34" s="13">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="C34" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D34" s="19" t="s">
+      <c r="C34" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" s="23" t="s">
         <v>152</v>
       </c>
-      <c r="E34" s="20"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="20"/>
-      <c r="H34" s="20"/>
-      <c r="I34" s="21"/>
-      <c r="J34" s="22" t="s">
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="25"/>
+      <c r="J34" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="K34" s="22" t="s">
+      <c r="K34" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="L34" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M34" s="18" t="s">
+      <c r="L34" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M34" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="N34" s="24">
+      <c r="N34" s="14">
         <v>1.4145000000000001</v>
       </c>
-      <c r="O34" s="25">
+      <c r="O34" s="15">
         <f t="shared" si="4"/>
         <v>7.0725000000000007</v>
       </c>
-      <c r="P34" s="27" t="s">
+      <c r="P34" s="17" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="35" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B35" s="23">
+      <c r="B35" s="13">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="C35" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D35" s="19" t="s">
+      <c r="C35" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="E35" s="20"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="20"/>
-      <c r="H35" s="20"/>
-      <c r="I35" s="21"/>
-      <c r="J35" s="22" t="s">
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="24"/>
+      <c r="I35" s="25"/>
+      <c r="J35" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="K35" s="22" t="s">
+      <c r="K35" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="L35" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M35" s="18" t="s">
+      <c r="L35" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M35" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="N35" s="24">
+      <c r="N35" s="14">
         <v>0.63300000000000001</v>
       </c>
-      <c r="O35" s="25">
+      <c r="O35" s="15">
         <f t="shared" si="4"/>
         <v>3.165</v>
       </c>
-      <c r="P35" s="27" t="s">
+      <c r="P35" s="17" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="36" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B36" s="23">
+      <c r="B36" s="13">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="C36" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D36" s="19" t="s">
+      <c r="C36" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="E36" s="20"/>
-      <c r="F36" s="20"/>
-      <c r="G36" s="20"/>
-      <c r="H36" s="20"/>
-      <c r="I36" s="21"/>
-      <c r="J36" s="22" t="s">
+      <c r="E36" s="24"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="24"/>
+      <c r="I36" s="25"/>
+      <c r="J36" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="K36" s="22" t="s">
+      <c r="K36" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="L36" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="M36" s="18" t="s">
+      <c r="L36" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="M36" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="N36" s="24">
+      <c r="N36" s="14">
         <v>4.3665000000000003</v>
       </c>
-      <c r="O36" s="25">
+      <c r="O36" s="15">
         <f t="shared" si="4"/>
         <v>21.832500000000003</v>
       </c>
-      <c r="P36" s="27" t="s">
+      <c r="P36" s="17" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="37" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="M37" s="28" t="s">
+      <c r="M37" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="N37" s="29"/>
+      <c r="N37" s="8"/>
       <c r="O37" s="3">
         <f>SUM(O4:O36)</f>
         <v>108.76499999999999</v>
@@ -2457,15 +2469,17 @@
       <c r="C38" t="s">
         <v>8</v>
       </c>
-      <c r="F38" s="12"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="12"/>
-      <c r="I38" s="13"/>
-      <c r="J38" s="13"/>
-      <c r="K38" s="13"/>
-      <c r="L38" s="11"/>
-      <c r="M38" s="9"/>
-      <c r="N38" s="10"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5"/>
+      <c r="I38" s="5"/>
+      <c r="J38" s="5"/>
+      <c r="K38" s="5"/>
+      <c r="L38" s="9"/>
+      <c r="M38" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="N38" s="30"/>
       <c r="O38" s="2"/>
     </row>
     <row r="39" spans="2:16" x14ac:dyDescent="0.2">
@@ -2482,36 +2496,76 @@
       <c r="J39" s="5"/>
       <c r="K39" s="5"/>
       <c r="L39" s="5"/>
-      <c r="M39" s="7" t="s">
+      <c r="M39" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="N39" s="7"/>
+      <c r="N39" s="32"/>
       <c r="O39" s="6">
         <f>O38+O37</f>
         <v>108.76499999999999</v>
       </c>
     </row>
     <row r="40" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="M40" s="30" t="s">
+      <c r="M40" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="O40" s="31">
+      <c r="O40" s="19">
         <f>O39/5</f>
         <v>21.752999999999997</v>
       </c>
     </row>
+    <row r="42" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="M42" t="s">
+        <v>164</v>
+      </c>
+      <c r="N42" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="43" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="M43" t="s">
+        <v>39</v>
+      </c>
+      <c r="N43" s="33">
+        <v>116.94</v>
+      </c>
+    </row>
+    <row r="44" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="M44" t="s">
+        <v>100</v>
+      </c>
+      <c r="N44" s="33">
+        <v>22.43</v>
+      </c>
+    </row>
+    <row r="45" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="M45" t="s">
+        <v>163</v>
+      </c>
+      <c r="N45" s="33">
+        <v>18.690000000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="N46" s="33">
+        <f>SUM(N43:N45)</f>
+        <v>158.06</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="D32:I32"/>
-    <mergeCell ref="D33:I33"/>
-    <mergeCell ref="D34:I34"/>
-    <mergeCell ref="D35:I35"/>
-    <mergeCell ref="D36:I36"/>
-    <mergeCell ref="D14:I14"/>
-    <mergeCell ref="D17:I17"/>
-    <mergeCell ref="D18:I18"/>
-    <mergeCell ref="D19:I19"/>
-    <mergeCell ref="D20:I20"/>
+    <mergeCell ref="M39:N39"/>
+    <mergeCell ref="D13:I13"/>
+    <mergeCell ref="D3:I3"/>
+    <mergeCell ref="D4:I4"/>
+    <mergeCell ref="D5:I5"/>
+    <mergeCell ref="D6:I6"/>
+    <mergeCell ref="D7:I7"/>
+    <mergeCell ref="D8:I8"/>
+    <mergeCell ref="D9:I9"/>
+    <mergeCell ref="D10:I10"/>
+    <mergeCell ref="D11:I11"/>
+    <mergeCell ref="D12:I12"/>
     <mergeCell ref="M38:N38"/>
     <mergeCell ref="D16:I16"/>
     <mergeCell ref="D15:I15"/>
@@ -2526,18 +2580,16 @@
     <mergeCell ref="D29:I29"/>
     <mergeCell ref="D30:I30"/>
     <mergeCell ref="D31:I31"/>
-    <mergeCell ref="D13:I13"/>
-    <mergeCell ref="D3:I3"/>
-    <mergeCell ref="D4:I4"/>
-    <mergeCell ref="D5:I5"/>
-    <mergeCell ref="D6:I6"/>
-    <mergeCell ref="D7:I7"/>
-    <mergeCell ref="D8:I8"/>
-    <mergeCell ref="D9:I9"/>
-    <mergeCell ref="D10:I10"/>
-    <mergeCell ref="D11:I11"/>
-    <mergeCell ref="D12:I12"/>
-    <mergeCell ref="M39:N39"/>
+    <mergeCell ref="D14:I14"/>
+    <mergeCell ref="D17:I17"/>
+    <mergeCell ref="D18:I18"/>
+    <mergeCell ref="D19:I19"/>
+    <mergeCell ref="D20:I20"/>
+    <mergeCell ref="D32:I32"/>
+    <mergeCell ref="D33:I33"/>
+    <mergeCell ref="D34:I34"/>
+    <mergeCell ref="D35:I35"/>
+    <mergeCell ref="D36:I36"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="P5" r:id="rId1" xr:uid="{5644B2BA-ED03-8440-9B66-CBBFBD5F9484}"/>

</xml_diff>

<commit_message>
Slight changes to schematic
</commit_message>
<xml_diff>
--- a/Charge_Indicator/BOM and Order Sheet/Order_Sheet.xlsx
+++ b/Charge_Indicator/BOM and Order Sheet/Order_Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nathanfikes/Documents/GitHub/AutoNav-Charge_Indicator-KiCad_Pcb/Charge_Indicator/BOM and Order Sheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9072578-7390-B146-93FF-E887100355D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DD79499-80EB-FF43-9C20-B2C223809897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11000" yWindow="680" windowWidth="19240" windowHeight="18020" xr2:uid="{F977D430-13CE-AD47-96E5-85BBB755CDD5}"/>
+    <workbookView xWindow="8320" yWindow="680" windowWidth="21920" windowHeight="17800" xr2:uid="{F977D430-13CE-AD47-96E5-85BBB755CDD5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -741,6 +741,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -749,6 +753,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -765,13 +772,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1132,14 +1132,14 @@
       <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="31" t="s">
+      <c r="D3" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
       <c r="J3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1173,14 +1173,14 @@
       <c r="C4" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="28"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="31"/>
       <c r="J4" s="10" t="s">
         <v>14</v>
       </c>
@@ -1213,14 +1213,14 @@
       <c r="C5" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="28"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="31"/>
       <c r="J5" s="10" t="s">
         <v>20</v>
       </c>
@@ -1252,14 +1252,14 @@
       <c r="C6" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="28"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="31"/>
       <c r="J6" s="10" t="s">
         <v>26</v>
       </c>
@@ -1291,14 +1291,14 @@
       <c r="C7" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="28"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="31"/>
       <c r="J7" s="10" t="s">
         <v>27</v>
       </c>
@@ -1330,14 +1330,14 @@
       <c r="C8" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="28"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="31"/>
       <c r="J8" s="10" t="s">
         <v>38</v>
       </c>
@@ -1369,14 +1369,14 @@
       <c r="C9" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="28"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="31"/>
       <c r="J9" s="10" t="s">
         <v>44</v>
       </c>
@@ -1408,14 +1408,14 @@
       <c r="C10" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="26" t="s">
+      <c r="D10" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="28"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="31"/>
       <c r="J10" s="10" t="s">
         <v>49</v>
       </c>
@@ -1447,14 +1447,14 @@
       <c r="C11" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="D11" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="28"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="31"/>
       <c r="J11" s="10" t="s">
         <v>55</v>
       </c>
@@ -1486,14 +1486,14 @@
       <c r="C12" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="25"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="27"/>
       <c r="J12" s="10" t="s">
         <v>59</v>
       </c>
@@ -1525,14 +1525,14 @@
       <c r="C13" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="25"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="27"/>
       <c r="J13" s="12" t="s">
         <v>61</v>
       </c>
@@ -1564,14 +1564,14 @@
       <c r="C14" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="D14" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="25"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="27"/>
       <c r="J14" s="10" t="s">
         <v>64</v>
       </c>
@@ -1603,14 +1603,14 @@
       <c r="C15" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="D15" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="25"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="27"/>
       <c r="J15" s="12" t="s">
         <v>68</v>
       </c>
@@ -1641,14 +1641,14 @@
       <c r="C16" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="23" t="s">
+      <c r="D16" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="25"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="27"/>
       <c r="J16" s="12" t="s">
         <v>73</v>
       </c>
@@ -1680,14 +1680,14 @@
       <c r="C17" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="29" t="s">
         <v>74</v>
       </c>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="28"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="31"/>
       <c r="J17" s="10" t="s">
         <v>77</v>
       </c>
@@ -1719,14 +1719,14 @@
       <c r="C18" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D18" s="26" t="s">
+      <c r="D18" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="28"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="31"/>
       <c r="J18" s="10" t="s">
         <v>80</v>
       </c>
@@ -1758,14 +1758,14 @@
       <c r="C19" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="D19" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="25"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="27"/>
       <c r="J19" s="12" t="s">
         <v>86</v>
       </c>
@@ -1797,14 +1797,14 @@
       <c r="C20" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="23" t="s">
+      <c r="D20" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="25"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="27"/>
       <c r="J20" s="12" t="s">
         <v>90</v>
       </c>
@@ -1836,14 +1836,14 @@
       <c r="C21" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="23" t="s">
+      <c r="D21" s="25" t="s">
         <v>96</v>
       </c>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="24"/>
-      <c r="I21" s="25"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="27"/>
       <c r="J21" s="10" t="s">
         <v>94</v>
       </c>
@@ -1875,14 +1875,14 @@
       <c r="C22" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="23" t="s">
+      <c r="D22" s="25" t="s">
         <v>98</v>
       </c>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24"/>
-      <c r="I22" s="25"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="26"/>
+      <c r="I22" s="27"/>
       <c r="J22" s="12" t="s">
         <v>99</v>
       </c>
@@ -1914,14 +1914,14 @@
       <c r="C23" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="23" t="s">
+      <c r="D23" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="25"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="27"/>
       <c r="J23" s="10" t="s">
         <v>105</v>
       </c>
@@ -1953,14 +1953,14 @@
       <c r="C24" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="26" t="s">
+      <c r="D24" s="29" t="s">
         <v>110</v>
       </c>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="27"/>
-      <c r="I24" s="28"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="31"/>
       <c r="J24" s="10" t="s">
         <v>108</v>
       </c>
@@ -1992,14 +1992,14 @@
       <c r="C25" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="26" t="s">
+      <c r="D25" s="29" t="s">
         <v>115</v>
       </c>
-      <c r="E25" s="27"/>
-      <c r="F25" s="27"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="27"/>
-      <c r="I25" s="28"/>
+      <c r="E25" s="30"/>
+      <c r="F25" s="30"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="30"/>
+      <c r="I25" s="31"/>
       <c r="J25" s="10" t="s">
         <v>113</v>
       </c>
@@ -2031,14 +2031,14 @@
       <c r="C26" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D26" s="23" t="s">
+      <c r="D26" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
-      <c r="H26" s="24"/>
-      <c r="I26" s="25"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="26"/>
+      <c r="H26" s="26"/>
+      <c r="I26" s="27"/>
       <c r="J26" s="10" t="s">
         <v>117</v>
       </c>
@@ -2070,14 +2070,14 @@
       <c r="C27" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D27" s="23" t="s">
+      <c r="D27" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="25"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="26"/>
+      <c r="I27" s="27"/>
       <c r="J27" s="12" t="s">
         <v>120</v>
       </c>
@@ -2109,14 +2109,14 @@
       <c r="C28" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D28" s="23" t="s">
+      <c r="D28" s="25" t="s">
         <v>125</v>
       </c>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="24"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="25"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="26"/>
+      <c r="H28" s="26"/>
+      <c r="I28" s="27"/>
       <c r="J28" s="10" t="s">
         <v>126</v>
       </c>
@@ -2148,14 +2148,14 @@
       <c r="C29" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D29" s="23" t="s">
+      <c r="D29" s="25" t="s">
         <v>129</v>
       </c>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="24"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="25"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="26"/>
+      <c r="H29" s="26"/>
+      <c r="I29" s="27"/>
       <c r="J29" s="12" t="s">
         <v>130</v>
       </c>
@@ -2187,14 +2187,14 @@
       <c r="C30" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D30" s="23" t="s">
+      <c r="D30" s="25" t="s">
         <v>133</v>
       </c>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
-      <c r="G30" s="24"/>
-      <c r="H30" s="24"/>
-      <c r="I30" s="25"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="27"/>
       <c r="J30" s="10" t="s">
         <v>134</v>
       </c>
@@ -2226,14 +2226,14 @@
       <c r="C31" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D31" s="26" t="s">
+      <c r="D31" s="29" t="s">
         <v>137</v>
       </c>
-      <c r="E31" s="27"/>
-      <c r="F31" s="27"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="28"/>
+      <c r="E31" s="30"/>
+      <c r="F31" s="30"/>
+      <c r="G31" s="30"/>
+      <c r="H31" s="30"/>
+      <c r="I31" s="31"/>
       <c r="J31" s="10" t="s">
         <v>138</v>
       </c>
@@ -2265,14 +2265,14 @@
       <c r="C32" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D32" s="23" t="s">
+      <c r="D32" s="25" t="s">
         <v>143</v>
       </c>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="24"/>
-      <c r="I32" s="25"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="26"/>
+      <c r="G32" s="26"/>
+      <c r="H32" s="26"/>
+      <c r="I32" s="27"/>
       <c r="J32" s="12">
         <v>1711725</v>
       </c>
@@ -2304,14 +2304,14 @@
       <c r="C33" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D33" s="23" t="s">
+      <c r="D33" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-      <c r="G33" s="24"/>
-      <c r="H33" s="24"/>
-      <c r="I33" s="25"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="26"/>
+      <c r="G33" s="26"/>
+      <c r="H33" s="26"/>
+      <c r="I33" s="27"/>
       <c r="J33" s="12" t="s">
         <v>147</v>
       </c>
@@ -2343,14 +2343,14 @@
       <c r="C34" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D34" s="23" t="s">
+      <c r="D34" s="25" t="s">
         <v>152</v>
       </c>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="24"/>
-      <c r="I34" s="25"/>
+      <c r="E34" s="26"/>
+      <c r="F34" s="26"/>
+      <c r="G34" s="26"/>
+      <c r="H34" s="26"/>
+      <c r="I34" s="27"/>
       <c r="J34" s="12" t="s">
         <v>150</v>
       </c>
@@ -2382,14 +2382,14 @@
       <c r="C35" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D35" s="23" t="s">
+      <c r="D35" s="25" t="s">
         <v>156</v>
       </c>
-      <c r="E35" s="24"/>
-      <c r="F35" s="24"/>
-      <c r="G35" s="24"/>
-      <c r="H35" s="24"/>
-      <c r="I35" s="25"/>
+      <c r="E35" s="26"/>
+      <c r="F35" s="26"/>
+      <c r="G35" s="26"/>
+      <c r="H35" s="26"/>
+      <c r="I35" s="27"/>
       <c r="J35" s="12" t="s">
         <v>155</v>
       </c>
@@ -2421,14 +2421,14 @@
       <c r="C36" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D36" s="23" t="s">
+      <c r="D36" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="E36" s="24"/>
-      <c r="F36" s="24"/>
-      <c r="G36" s="24"/>
-      <c r="H36" s="24"/>
-      <c r="I36" s="25"/>
+      <c r="E36" s="26"/>
+      <c r="F36" s="26"/>
+      <c r="G36" s="26"/>
+      <c r="H36" s="26"/>
+      <c r="I36" s="27"/>
       <c r="J36" s="12" t="s">
         <v>158</v>
       </c>
@@ -2476,10 +2476,10 @@
       <c r="J38" s="5"/>
       <c r="K38" s="5"/>
       <c r="L38" s="9"/>
-      <c r="M38" s="29" t="s">
+      <c r="M38" s="32" t="s">
         <v>162</v>
       </c>
-      <c r="N38" s="30"/>
+      <c r="N38" s="33"/>
       <c r="O38" s="2"/>
     </row>
     <row r="39" spans="2:16" x14ac:dyDescent="0.2">
@@ -2496,10 +2496,10 @@
       <c r="J39" s="5"/>
       <c r="K39" s="5"/>
       <c r="L39" s="5"/>
-      <c r="M39" s="32" t="s">
+      <c r="M39" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="N39" s="32"/>
+      <c r="N39" s="24"/>
       <c r="O39" s="6">
         <f>O38+O37</f>
         <v>108.76499999999999</v>
@@ -2514,19 +2514,21 @@
         <v>21.752999999999997</v>
       </c>
     </row>
+    <row r="41" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="M41" t="s">
+        <v>165</v>
+      </c>
+    </row>
     <row r="42" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="M42" t="s">
+      <c r="M42" s="18" t="s">
         <v>164</v>
-      </c>
-      <c r="N42" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="43" spans="2:16" x14ac:dyDescent="0.2">
       <c r="M43" t="s">
         <v>39</v>
       </c>
-      <c r="N43" s="33">
+      <c r="N43" s="23">
         <v>116.94</v>
       </c>
     </row>
@@ -2534,7 +2536,7 @@
       <c r="M44" t="s">
         <v>100</v>
       </c>
-      <c r="N44" s="33">
+      <c r="N44" s="23">
         <v>22.43</v>
       </c>
     </row>
@@ -2542,18 +2544,38 @@
       <c r="M45" t="s">
         <v>163</v>
       </c>
-      <c r="N45" s="33">
+      <c r="N45" s="23">
         <v>18.690000000000001</v>
       </c>
     </row>
     <row r="46" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="N46" s="33">
+      <c r="N46" s="23">
         <f>SUM(N43:N45)</f>
         <v>158.06</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="36">
+    <mergeCell ref="D32:I32"/>
+    <mergeCell ref="D33:I33"/>
+    <mergeCell ref="D34:I34"/>
+    <mergeCell ref="D35:I35"/>
+    <mergeCell ref="D36:I36"/>
+    <mergeCell ref="D14:I14"/>
+    <mergeCell ref="D17:I17"/>
+    <mergeCell ref="D18:I18"/>
+    <mergeCell ref="D19:I19"/>
+    <mergeCell ref="D20:I20"/>
+    <mergeCell ref="D27:I27"/>
+    <mergeCell ref="D28:I28"/>
+    <mergeCell ref="D29:I29"/>
+    <mergeCell ref="D30:I30"/>
+    <mergeCell ref="D31:I31"/>
+    <mergeCell ref="D22:I22"/>
+    <mergeCell ref="D23:I23"/>
+    <mergeCell ref="D24:I24"/>
+    <mergeCell ref="D25:I25"/>
+    <mergeCell ref="D26:I26"/>
     <mergeCell ref="M39:N39"/>
     <mergeCell ref="D13:I13"/>
     <mergeCell ref="D3:I3"/>
@@ -2570,26 +2592,6 @@
     <mergeCell ref="D16:I16"/>
     <mergeCell ref="D15:I15"/>
     <mergeCell ref="D21:I21"/>
-    <mergeCell ref="D22:I22"/>
-    <mergeCell ref="D23:I23"/>
-    <mergeCell ref="D24:I24"/>
-    <mergeCell ref="D25:I25"/>
-    <mergeCell ref="D26:I26"/>
-    <mergeCell ref="D27:I27"/>
-    <mergeCell ref="D28:I28"/>
-    <mergeCell ref="D29:I29"/>
-    <mergeCell ref="D30:I30"/>
-    <mergeCell ref="D31:I31"/>
-    <mergeCell ref="D14:I14"/>
-    <mergeCell ref="D17:I17"/>
-    <mergeCell ref="D18:I18"/>
-    <mergeCell ref="D19:I19"/>
-    <mergeCell ref="D20:I20"/>
-    <mergeCell ref="D32:I32"/>
-    <mergeCell ref="D33:I33"/>
-    <mergeCell ref="D34:I34"/>
-    <mergeCell ref="D35:I35"/>
-    <mergeCell ref="D36:I36"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="P5" r:id="rId1" xr:uid="{5644B2BA-ED03-8440-9B66-CBBFBD5F9484}"/>

</xml_diff>